<commit_message>
Marked as final and Digitally Signed
</commit_message>
<xml_diff>
--- a/data/Brokerage.xlsx
+++ b/data/Brokerage.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pmoor\Cursor\tech_drawdown\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pmoor\bob\tech_drawdown\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE662C75-1DDF-4D62-AB46-11E7DF3FA29E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41486532-1B71-4538-876E-554A5CF92EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0513BBD6-4D7E-4578-96A4-088A6094004C}"/>
   </bookViews>
@@ -988,4 +988,169 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=_xmlsignatures/sig1.xml><?xml version="1.0" encoding="utf-8"?>
+<Signature xmlns="http://www.w3.org/2000/09/xmldsig#" Id="idPackageSignature">
+  <SignedInfo>
+    <CanonicalizationMethod Algorithm="http://www.w3.org/TR/2001/REC-xml-c14n-20010315"/>
+    <SignatureMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#ecdsa-sha384"/>
+    <Reference Type="http://www.w3.org/2000/09/xmldsig#Object" URI="#idPackageObject">
+      <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+      <DigestValue>6h604aUb6Tf/A7r7MC+rPspdm0lFTPH0Eb+44sNxWI7uDYuogsokAh1QkDmxMIHB</DigestValue>
+    </Reference>
+    <Reference Type="http://www.w3.org/2000/09/xmldsig#Object" URI="#idOfficeObject">
+      <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+      <DigestValue>ymV95A8Q+Bxp8EWZ/J6n/k0jnCZie3pua+KZnDPPxnW4WX+LPNnIsJGXkEdwKCiv</DigestValue>
+    </Reference>
+    <Reference Type="http://uri.etsi.org/01903#SignedProperties" URI="#idSignedProperties">
+      <Transforms>
+        <Transform Algorithm="http://www.w3.org/TR/2001/REC-xml-c14n-20010315"/>
+      </Transforms>
+      <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+      <DigestValue>6lCueSUPG2q7Qh8MvJuin/pp9D3lWLwLuutRBnv28/6IIgsFLR1577GhPuYyUhU/</DigestValue>
+    </Reference>
+  </SignedInfo>
+  <SignatureValue>mWtq4HWdczVeawgwoLsFHWKPfTjLwifDD2XlhBl+86Pa2lx2Moe5gWfqidQmaZHMVym0aGIuyjDZ
+bYTp5Rip1/gC1opagmVRbYX2WNVpRh0wNyoBt1YyWipZFwaLBf6H</SignatureValue>
+  <KeyInfo>
+    <X509Data>
+      <X509Certificate>MIIBkTCCARagAwIBAgIJAPdIHSGNfZuUMAoGCCqGSM49BAMDMC8xLTArBgNVBAMTJGNhYTIyY2YxLWMxM2YtNDM3Yy1iYWZkLWFhNjM5MjU5MDkzMTAeFw0yNjAzMDgwMTU2MzlaFw0yNzAzMDgxMzU2MzlaMC8xLTArBgNVBAMTJGNhYTIyY2YxLWMxM2YtNDM3Yy1iYWZkLWFhNjM5MjU5MDkzMTB2MBAGByqGSM49AgEGBSuBBAAiA2IABNp6f9pfSrQcXKO+mGODiKCBvrFCgM6z6svOeFdn85eIZkMNYGiGy4qv372dsw6lUyYdMetE51bq0gc2taRfqpv74xATA8+srJCgSRF8wKRuy54sgtL8WciTs1VhOPHsaTAKBggqhkjOPQQDAwNpADBmAjEA5hZTKtauY9KNCFdXK5ZSsXmnIrEb3vm1m+GkTPdKWTDFsKMxe03DPvyHL6v5vvpnAjEAsDyuNkP5luWjdar8Nfd6yIN8WevzfJxqjLpxnT0OFiseNRTv1Xfsu9jmilU9jePZ</X509Certificate>
+    </X509Data>
+  </KeyInfo>
+  <Object Id="idPackageObject">
+    <Manifest>
+      <Reference URI="/_rels/.rels?ContentType=application/vnd.openxmlformats-package.relationships+xml">
+        <Transforms>
+          <Transform Algorithm="http://schemas.openxmlformats.org/package/2006/RelationshipTransform">
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId1"/>
+          </Transform>
+          <Transform Algorithm="http://www.w3.org/TR/2001/REC-xml-c14n-20010315"/>
+        </Transforms>
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>Mf2/mKvHoEm+XQe0V5FnG8+mCC19i1rJCIQNslrm4nmnCLDlck67lEpi2D8bIPxk</DigestValue>
+      </Reference>
+      <Reference URI="/xl/_rels/workbook.xml.rels?ContentType=application/vnd.openxmlformats-package.relationships+xml">
+        <Transforms>
+          <Transform Algorithm="http://schemas.openxmlformats.org/package/2006/RelationshipTransform">
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId4"/>
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId3"/>
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId2"/>
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId1"/>
+            <mdssi:RelationshipReference xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature" SourceId="rId5"/>
+          </Transform>
+          <Transform Algorithm="http://www.w3.org/TR/2001/REC-xml-c14n-20010315"/>
+        </Transforms>
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>LZIEeOv4vR2ZK8iFsNQ1ROaEBVtZGseXVpbngCcQvfVee5tEWhUVJmcRKe06dVyc</DigestValue>
+      </Reference>
+      <Reference URI="/xl/calcChain.xml?ContentType=application/vnd.openxmlformats-officedocument.spreadsheetml.calcChain+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>LH12pjyXI/tMF87lJrkUMWwJ+vcVwDUgACPDlicHhK3qMVFxTgT9teb+GZyIrQd9</DigestValue>
+      </Reference>
+      <Reference URI="/xl/sharedStrings.xml?ContentType=application/vnd.openxmlformats-officedocument.spreadsheetml.sharedStrings+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>psm6lHebfiUmmG1PwqaV6B8ygM4aBXVyIKO2RgilIGSC1mNVFH7qSGuikSBeVa2e</DigestValue>
+      </Reference>
+      <Reference URI="/xl/styles.xml?ContentType=application/vnd.openxmlformats-officedocument.spreadsheetml.styles+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>CTRHJKTQugFFFi7l7rZ2hmfRbniGxZDnDBGKLG+pBoPCWUCR1FJuytfJ5mmuKopK</DigestValue>
+      </Reference>
+      <Reference URI="/xl/theme/theme1.xml?ContentType=application/vnd.openxmlformats-officedocument.theme+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>nxbunxDMsQvWp5VIFRdAnfkbWkPSPb6QJ26j1oQkf6LHTbWnrPr57N4d59q4IAIr</DigestValue>
+      </Reference>
+      <Reference URI="/xl/workbook.xml?ContentType=application/vnd.openxmlformats-officedocument.spreadsheetml.sheet.main+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>Ge6OKzx9V0RgICpEpG4junacbC5Nd1suuYEXTVgkWrh1ofbu2UAjbN6pmwxuwTJt</DigestValue>
+      </Reference>
+      <Reference URI="/xl/worksheets/sheet1.xml?ContentType=application/vnd.openxmlformats-officedocument.spreadsheetml.worksheet+xml">
+        <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+        <DigestValue>6T0yuvgFKo+TDdqOaB0+VZJu2gY0/DC6XjLS5Px9Niqz9AcqBfsYdDfxGy+XW/W9</DigestValue>
+      </Reference>
+    </Manifest>
+    <SignatureProperties>
+      <SignatureProperty Id="idSignatureTime" Target="#idPackageSignature">
+        <mdssi:SignatureTime xmlns:mdssi="http://schemas.openxmlformats.org/package/2006/digital-signature">
+          <mdssi:Format>YYYY-MM-DDThh:mm:ssTZD</mdssi:Format>
+          <mdssi:Value>2026-08-29T16:42:13Z</mdssi:Value>
+        </mdssi:SignatureTime>
+      </SignatureProperty>
+    </SignatureProperties>
+  </Object>
+  <Object Id="idOfficeObject">
+    <SignatureProperties>
+      <SignatureProperty Id="idOfficeV1Details" Target="#idPackageSignature">
+        <SignatureInfoV1 xmlns="http://schemas.microsoft.com/office/2006/digsig">
+          <SetupID/>
+          <SignatureText/>
+          <SignatureImage/>
+          <SignatureComments>Submission for IBM review</SignatureComments>
+          <WindowsVersion>10.0</WindowsVersion>
+          <OfficeVersion>16.0.20326/27</OfficeVersion>
+          <ApplicationVersion>16.0.20326</ApplicationVersion>
+          <Monitors>1</Monitors>
+          <HorizontalResolution>1920</HorizontalResolution>
+          <VerticalResolution>1080</VerticalResolution>
+          <ColorDepth>32</ColorDepth>
+          <SignatureProviderId>{00000000-0000-0000-0000-000000000000}</SignatureProviderId>
+          <SignatureProviderUrl/>
+          <SignatureProviderDetails>9</SignatureProviderDetails>
+          <SignatureType>1</SignatureType>
+        </SignatureInfoV1>
+        <SignatureInfoV2 xmlns="http://schemas.microsoft.com/office/2006/digsig">
+          <Address1/>
+          <Address2/>
+        </SignatureInfoV2>
+      </SignatureProperty>
+    </SignatureProperties>
+  </Object>
+  <Object>
+    <xd:QualifyingProperties xmlns:xd="http://uri.etsi.org/01903/v1.3.2#" Target="#idPackageSignature">
+      <xd:SignedProperties Id="idSignedProperties">
+        <xd:SignedSignatureProperties>
+          <xd:SigningTime>2026-08-29T16:42:13Z</xd:SigningTime>
+          <xd:SigningCertificate>
+            <xd:Cert>
+              <xd:CertDigest>
+                <DigestMethod Algorithm="http://www.w3.org/2001/04/xmldsig-more#sha384"/>
+                <DigestValue>AAGwLZ0Mju8BR7lCmJFzSejv/Gfu6+ToSzLGusuNTd9Nzga1YrQDdyDar9Vdx84e</DigestValue>
+              </xd:CertDigest>
+              <xd:IssuerSerial>
+                <X509IssuerName>CN=caa22cf1-c13f-437c-bafd-aa6392590931</X509IssuerName>
+                <X509SerialNumber>17818523955636312980</X509SerialNumber>
+              </xd:IssuerSerial>
+            </xd:Cert>
+          </xd:SigningCertificate>
+          <xd:SignaturePolicyIdentifier>
+            <xd:SignaturePolicyImplied/>
+          </xd:SignaturePolicyIdentifier>
+          <xd:SignatureProductionPlace>
+            <xd:City/>
+            <xd:StateOrProvince/>
+            <xd:PostalCode/>
+            <xd:CountryName/>
+          </xd:SignatureProductionPlace>
+          <xd:SignerRole>
+            <xd:ClaimedRoles>
+              <xd:ClaimedRole>Author</xd:ClaimedRole>
+            </xd:ClaimedRoles>
+          </xd:SignerRole>
+        </xd:SignedSignatureProperties>
+        <xd:SignedDataObjectProperties>
+          <xd:CommitmentTypeIndication>
+            <xd:CommitmentTypeId>
+              <xd:Identifier>http://uri.etsi.org/01903/v1.2.2#ProofOfOrigin</xd:Identifier>
+              <xd:Description>Created and approved this document</xd:Description>
+            </xd:CommitmentTypeId>
+            <xd:AllSignedDataObjects/>
+            <xd:CommitmentTypeQualifiers>
+              <xd:CommitmentTypeQualifier>Submission for IBM review</xd:CommitmentTypeQualifier>
+            </xd:CommitmentTypeQualifiers>
+          </xd:CommitmentTypeIndication>
+        </xd:SignedDataObjectProperties>
+      </xd:SignedProperties>
+    </xd:QualifyingProperties>
+  </Object>
+</Signature>
 </file>
</xml_diff>